<commit_message>
Update Quote Bank CMS to use Snippet categories dynamically
</commit_message>
<xml_diff>
--- a/Quote_Bank_Resources_Manager/categories.xlsx
+++ b/Quote_Bank_Resources_Manager/categories.xlsx
@@ -1,35 +1,104 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\RONE_MentorOS\Quote_Bank_Resources_Manager\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD5138C7-AE4A-461C-B5B4-059ED455AAFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Categories" sheetId="1" r:id="rId1"/>
+    <sheet name="Metadata" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Good Introduction</t>
+  </si>
+  <si>
+    <t>Good Body / Arguments</t>
+  </si>
+  <si>
+    <t>Good Conclusion</t>
+  </si>
+  <si>
+    <t>Data &amp; Facts Usage</t>
+  </si>
+  <si>
+    <t>Diagrams &amp; Maps</t>
+  </si>
+  <si>
+    <t>Presentation / Handwriting</t>
+  </si>
+  <si>
+    <t>Areas of Improvement</t>
+  </si>
+  <si>
+    <t>Rank / Name</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Paper</t>
+  </si>
+  <si>
+    <t>Rank 1 - Shruti Sharma</t>
+  </si>
+  <si>
+    <t>GS Paper 1</t>
+  </si>
+  <si>
+    <t>Rank 2 - Ankita Agarwal</t>
+  </si>
+  <si>
+    <t>GS Paper 2</t>
+  </si>
+  <si>
+    <t>Rank 3 - Gamini Singla</t>
+  </si>
+  <si>
+    <t>GS Paper 3</t>
+  </si>
+  <si>
+    <t>GS Paper 4</t>
+  </si>
+  <si>
+    <t>Essay</t>
+  </si>
+  <si>
+    <t>Optional</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -48,80 +117,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -409,68 +419,51 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Good Introduction</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Good Body / Arguments</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Good Conclusion</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Data &amp; Facts Usage</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Diagrams &amp; Maps</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Presentation / Handwriting</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Areas of Improvement</t>
-        </is>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -479,101 +472,72 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Rank / Name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Paper</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Rank 1 - Shruti Sharma</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2">
         <v>2023</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GS Paper 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Rank 2 - Ankita Agarwal</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3">
         <v>2024</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GS Paper 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Rank 3 - Gamini Singla</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4">
         <v>2025</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GS Paper 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>GS Paper 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Essay</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update page titles to RONE MentorOS
</commit_message>
<xml_diff>
--- a/Quote_Bank_Resources_Manager/categories.xlsx
+++ b/Quote_Bank_Resources_Manager/categories.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\RONE_MentorOS\Quote_Bank_Resources_Manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD5138C7-AE4A-461C-B5B4-059ED455AAFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC5BE9AE-CF37-400A-91D7-9A51054437CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,32 +21,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Category</t>
   </si>
   <si>
-    <t>Good Introduction</t>
-  </si>
-  <si>
-    <t>Good Body / Arguments</t>
-  </si>
-  <si>
-    <t>Good Conclusion</t>
-  </si>
-  <si>
-    <t>Data &amp; Facts Usage</t>
-  </si>
-  <si>
-    <t>Diagrams &amp; Maps</t>
-  </si>
-  <si>
-    <t>Presentation / Handwriting</t>
-  </si>
-  <si>
-    <t>Areas of Improvement</t>
-  </si>
-  <si>
     <t>Rank / Name</t>
   </si>
   <si>
@@ -81,6 +60,21 @@
   </si>
   <si>
     <t>Optional</t>
+  </si>
+  <si>
+    <t>⚖️ Ethics</t>
+  </si>
+  <si>
+    <t>🧠 Thinkers</t>
+  </si>
+  <si>
+    <t>🏛️ Gov</t>
+  </si>
+  <si>
+    <t>👥 Society</t>
+  </si>
+  <si>
+    <t>💼 Public Service</t>
   </si>
 </sst>
 </file>
@@ -420,10 +414,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -433,37 +428,27 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -483,61 +468,61 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B2">
         <v>2023</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B3">
         <v>2024</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B4">
         <v>2025</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Initial commit for new website
</commit_message>
<xml_diff>
--- a/Quote_Bank_Resources_Manager/categories.xlsx
+++ b/Quote_Bank_Resources_Manager/categories.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\RONE_MentorOS\Quote_Bank_Resources_Manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC5BE9AE-CF37-400A-91D7-9A51054437CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCDB21C9-287C-426C-AEAC-A30723984CD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>Category</t>
   </si>
@@ -41,40 +41,40 @@
     <t>GS Paper 1</t>
   </si>
   <si>
-    <t>Rank 2 - Ankita Agarwal</t>
-  </si>
-  <si>
     <t>GS Paper 2</t>
   </si>
   <si>
-    <t>Rank 3 - Gamini Singla</t>
-  </si>
-  <si>
     <t>GS Paper 3</t>
   </si>
   <si>
-    <t>GS Paper 4</t>
-  </si>
-  <si>
     <t>Essay</t>
   </si>
   <si>
-    <t>Optional</t>
-  </si>
-  <si>
-    <t>⚖️ Ethics</t>
-  </si>
-  <si>
-    <t>🧠 Thinkers</t>
-  </si>
-  <si>
-    <t>🏛️ Gov</t>
-  </si>
-  <si>
-    <t>👥 Society</t>
-  </si>
-  <si>
-    <t>💼 Public Service</t>
+    <t>⚖️Ethics</t>
+  </si>
+  <si>
+    <t>🧠Thinkers</t>
+  </si>
+  <si>
+    <t>🏛️Gov</t>
+  </si>
+  <si>
+    <t>👥Society</t>
+  </si>
+  <si>
+    <t>💼Public Service</t>
+  </si>
+  <si>
+    <t>Ethics</t>
+  </si>
+  <si>
+    <t>Thinkers</t>
+  </si>
+  <si>
+    <t>Gov</t>
+  </si>
+  <si>
+    <t>PUB ADD</t>
   </si>
 </sst>
 </file>
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -428,27 +428,42 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -489,40 +504,34 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
       <c r="B3">
         <v>2024</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
       <c r="B4">
         <v>2025</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UI: hide categorize accordion inside sync config and remove duplicate categories
</commit_message>
<xml_diff>
--- a/Quote_Bank_Resources_Manager/categories.xlsx
+++ b/Quote_Bank_Resources_Manager/categories.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\RONE_MentorOS\Quote_Bank_Resources_Manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCDB21C9-287C-426C-AEAC-A30723984CD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAB1A88D-91BE-4CD6-8AF3-CB7E15989123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
   <si>
     <t>Category</t>
   </si>
@@ -35,12 +35,6 @@
     <t>Paper</t>
   </si>
   <si>
-    <t>Rank 1 - Shruti Sharma</t>
-  </si>
-  <si>
-    <t>GS Paper 1</t>
-  </si>
-  <si>
     <t>GS Paper 2</t>
   </si>
   <si>
@@ -75,19 +69,130 @@
   </si>
   <si>
     <t>PUB ADD</t>
+  </si>
+  <si>
+    <t>Rank 1 shruti sharma</t>
+  </si>
+  <si>
+    <t>Rank 111 kashish kalra</t>
+  </si>
+  <si>
+    <t>Rank 156 zinnia aurora</t>
+  </si>
+  <si>
+    <t>Rank 210 sania seervi</t>
+  </si>
+  <si>
+    <t>Rank 37 shobhika pathak</t>
+  </si>
+  <si>
+    <t>Rank 50 k n chandana jahnavi</t>
+  </si>
+  <si>
+    <t>Rank 9 nausheen</t>
+  </si>
+  <si>
+    <t>Rank 289 chandar prabha sharma</t>
+  </si>
+  <si>
+    <t>Rank 399 oishee mandal</t>
+  </si>
+  <si>
+    <t>Rank 100 vijeta b hosamani</t>
+  </si>
+  <si>
+    <t>Rank 127 aditi upadhyay</t>
+  </si>
+  <si>
+    <t>Rank 189 poorva agrawal</t>
+  </si>
+  <si>
+    <t>Rank 194 aditi yadav</t>
+  </si>
+  <si>
+    <t>Rank 199 tripti kalhans</t>
+  </si>
+  <si>
+    <t>Rank 204 shubhra panda</t>
+  </si>
+  <si>
+    <t>Rank 99 annapurna singh</t>
+  </si>
+  <si>
+    <t>Rank 25 ritika verma</t>
+  </si>
+  <si>
+    <t>Rank 26 rupal rana</t>
+  </si>
+  <si>
+    <t>Rank 36 ayushi pradhan</t>
+  </si>
+  <si>
+    <t>Rank 39 deepti rohilla</t>
+  </si>
+  <si>
+    <t>RANK 51 RAJPUT NEHA UDDHAVSINGH</t>
+  </si>
+  <si>
+    <t>RANK 17 SWATI SHARMA</t>
+  </si>
+  <si>
+    <t>RANK 61 KHUSHHALI SOLANKI</t>
+  </si>
+  <si>
+    <t>RANK 65 CHHAYA SINGH</t>
+  </si>
+  <si>
+    <t>RANK 80 GARIMA MUNDRA</t>
+  </si>
+  <si>
+    <t>RANK 18 WARDAH KHAN</t>
+  </si>
+  <si>
+    <t>RANK 263 Girisha Chaudhary</t>
+  </si>
+  <si>
+    <t>RANK 1 Shakti Dubey</t>
+  </si>
+  <si>
+    <t>RANK 189 ANUPRIYA RAI</t>
+  </si>
+  <si>
+    <t>RANK 40 IRAM CHOUDHARY</t>
+  </si>
+  <si>
+    <t>RANK 7 AAYUSHI BANSAL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Mistral"/>
+      <family val="4"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Mistral"/>
+      <family val="4"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Mistral"/>
+      <family val="4"/>
     </font>
   </fonts>
   <fills count="2">
@@ -110,8 +215,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -428,42 +538,42 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -473,65 +583,219 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35" style="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="1">
+        <v>2021</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2022</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="1">
         <v>2023</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="1">
         <v>2024</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B4">
-        <v>2025</v>
-      </c>
-      <c r="C4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C7" t="s">
-        <v>17</v>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="21.75" x14ac:dyDescent="0.4">
+      <c r="A23" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Front Page Premium Redesign
</commit_message>
<xml_diff>
--- a/Quote_Bank_Resources_Manager/categories.xlsx
+++ b/Quote_Bank_Resources_Manager/categories.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\RONE_MentorOS\Quote_Bank_Resources_Manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAB1A88D-91BE-4CD6-8AF3-CB7E15989123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E4FCF9-5A34-4512-AB9E-25C2B76F2229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="47">
   <si>
     <t>Category</t>
   </si>
@@ -226,7 +226,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -659,7 +670,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7" s="1">
         <v>2026</v>
@@ -670,135 +681,136 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="21.75" x14ac:dyDescent="0.4">
-      <c r="A23" s="3" t="s">
+    <row r="22" spans="1:1" ht="21.75" x14ac:dyDescent="0.4">
+      <c r="A22" s="3" t="s">
         <v>36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" s="1" t="s">
         <v>46</v>
       </c>
     </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C33"/>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:A32 A34:A1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
remove: decorative icon grid from Quote Bank header
</commit_message>
<xml_diff>
--- a/Quote_Bank_Resources_Manager/categories.xlsx
+++ b/Quote_Bank_Resources_Manager/categories.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\RONE_MentorOS\Quote_Bank_Resources_Manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E4FCF9-5A34-4512-AB9E-25C2B76F2229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7891530-B71F-4375-B810-4B65D453CBD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -535,7 +535,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -562,28 +562,28 @@
         <v>14</v>
       </c>
     </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+    </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: prompt user for custom snippet name instead of random timestamp
</commit_message>
<xml_diff>
--- a/Quote_Bank_Resources_Manager/categories.xlsx
+++ b/Quote_Bank_Resources_Manager/categories.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\RONE_MentorOS\Quote_Bank_Resources_Manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7891530-B71F-4375-B810-4B65D453CBD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02188982-B9EE-43BF-98C8-755E64A5694A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="51">
   <si>
     <t>Category</t>
   </si>
@@ -162,6 +162,18 @@
   </si>
   <si>
     <t>RANK 7 AAYUSHI BANSAL</t>
+  </si>
+  <si>
+    <t>Theory Answers</t>
+  </si>
+  <si>
+    <t>Case Studies</t>
+  </si>
+  <si>
+    <t>Introductions</t>
+  </si>
+  <si>
+    <t>Conclusions</t>
   </si>
 </sst>
 </file>
@@ -535,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -585,6 +597,26 @@
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UI Updates: Add premium favicon, fix Ranker's Root folder ID, update dashboard layout
</commit_message>
<xml_diff>
--- a/Quote_Bank_Resources_Manager/categories.xlsx
+++ b/Quote_Bank_Resources_Manager/categories.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\RONE_MentorOS\Quote_Bank_Resources_Manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02188982-B9EE-43BF-98C8-755E64A5694A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0223AE4E-91D1-46B1-8A65-3E2F8469EA23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
   <si>
     <t>Category</t>
   </si>
@@ -44,21 +44,6 @@
     <t>Essay</t>
   </si>
   <si>
-    <t>⚖️Ethics</t>
-  </si>
-  <si>
-    <t>🧠Thinkers</t>
-  </si>
-  <si>
-    <t>🏛️Gov</t>
-  </si>
-  <si>
-    <t>👥Society</t>
-  </si>
-  <si>
-    <t>💼Public Service</t>
-  </si>
-  <si>
     <t>Ethics</t>
   </si>
   <si>
@@ -71,99 +56,6 @@
     <t>PUB ADD</t>
   </si>
   <si>
-    <t>Rank 1 shruti sharma</t>
-  </si>
-  <si>
-    <t>Rank 111 kashish kalra</t>
-  </si>
-  <si>
-    <t>Rank 156 zinnia aurora</t>
-  </si>
-  <si>
-    <t>Rank 210 sania seervi</t>
-  </si>
-  <si>
-    <t>Rank 37 shobhika pathak</t>
-  </si>
-  <si>
-    <t>Rank 50 k n chandana jahnavi</t>
-  </si>
-  <si>
-    <t>Rank 9 nausheen</t>
-  </si>
-  <si>
-    <t>Rank 289 chandar prabha sharma</t>
-  </si>
-  <si>
-    <t>Rank 399 oishee mandal</t>
-  </si>
-  <si>
-    <t>Rank 100 vijeta b hosamani</t>
-  </si>
-  <si>
-    <t>Rank 127 aditi upadhyay</t>
-  </si>
-  <si>
-    <t>Rank 189 poorva agrawal</t>
-  </si>
-  <si>
-    <t>Rank 194 aditi yadav</t>
-  </si>
-  <si>
-    <t>Rank 199 tripti kalhans</t>
-  </si>
-  <si>
-    <t>Rank 204 shubhra panda</t>
-  </si>
-  <si>
-    <t>Rank 99 annapurna singh</t>
-  </si>
-  <si>
-    <t>Rank 25 ritika verma</t>
-  </si>
-  <si>
-    <t>Rank 26 rupal rana</t>
-  </si>
-  <si>
-    <t>Rank 36 ayushi pradhan</t>
-  </si>
-  <si>
-    <t>Rank 39 deepti rohilla</t>
-  </si>
-  <si>
-    <t>RANK 51 RAJPUT NEHA UDDHAVSINGH</t>
-  </si>
-  <si>
-    <t>RANK 17 SWATI SHARMA</t>
-  </si>
-  <si>
-    <t>RANK 61 KHUSHHALI SOLANKI</t>
-  </si>
-  <si>
-    <t>RANK 65 CHHAYA SINGH</t>
-  </si>
-  <si>
-    <t>RANK 80 GARIMA MUNDRA</t>
-  </si>
-  <si>
-    <t>RANK 18 WARDAH KHAN</t>
-  </si>
-  <si>
-    <t>RANK 263 Girisha Chaudhary</t>
-  </si>
-  <si>
-    <t>RANK 1 Shakti Dubey</t>
-  </si>
-  <si>
-    <t>RANK 189 ANUPRIYA RAI</t>
-  </si>
-  <si>
-    <t>RANK 40 IRAM CHOUDHARY</t>
-  </si>
-  <si>
-    <t>RANK 7 AAYUSHI BANSAL</t>
-  </si>
-  <si>
     <t>Theory Answers</t>
   </si>
   <si>
@@ -174,6 +66,108 @@
   </si>
   <si>
     <t>Conclusions</t>
+  </si>
+  <si>
+    <t>Society</t>
+  </si>
+  <si>
+    <t>Public Service</t>
+  </si>
+  <si>
+    <t>GS Paper 1</t>
+  </si>
+  <si>
+    <t>rank 1 shruti sharma</t>
+  </si>
+  <si>
+    <t>rank 111 kashish kalra</t>
+  </si>
+  <si>
+    <t>rank 156 zinnia aurora</t>
+  </si>
+  <si>
+    <t>rank 210 sania seervi</t>
+  </si>
+  <si>
+    <t>rank 37 shobhika pathak</t>
+  </si>
+  <si>
+    <t>rank 50 k n chandana jahnavi</t>
+  </si>
+  <si>
+    <t>rank 9 nausheen</t>
+  </si>
+  <si>
+    <t>rank 289 chandar prabha sharma</t>
+  </si>
+  <si>
+    <t>rank 399 oishee mandal</t>
+  </si>
+  <si>
+    <t>rank 100 vijeta b hosamani</t>
+  </si>
+  <si>
+    <t>rank 127 aditi upadhyay</t>
+  </si>
+  <si>
+    <t>rank 189 poorva agrawal</t>
+  </si>
+  <si>
+    <t>rank 194 aditi yadav</t>
+  </si>
+  <si>
+    <t>rank 199 tripti kalhans</t>
+  </si>
+  <si>
+    <t>rank 204 shubhra panda</t>
+  </si>
+  <si>
+    <t>rank 99 annapurna singh</t>
+  </si>
+  <si>
+    <t>rank 25 ritika verma</t>
+  </si>
+  <si>
+    <t>rank 26 rupal rana</t>
+  </si>
+  <si>
+    <t>rank 36 ayushi pradhan</t>
+  </si>
+  <si>
+    <t>rank 39 deepti rohilla</t>
+  </si>
+  <si>
+    <t>rank 51 rajput neha uddhavsingh</t>
+  </si>
+  <si>
+    <t>rank 17 swati sharma</t>
+  </si>
+  <si>
+    <t>rank 61 khushhali solanki</t>
+  </si>
+  <si>
+    <t>rank 65 chhaya singh</t>
+  </si>
+  <si>
+    <t>rank 80 garima mundra</t>
+  </si>
+  <si>
+    <t>rank 18 wardah khan</t>
+  </si>
+  <si>
+    <t>rank 263 girisha chaudhary</t>
+  </si>
+  <si>
+    <t>rank 1 shakti dubey</t>
+  </si>
+  <si>
+    <t>rank 189 anupriya rai</t>
+  </si>
+  <si>
+    <t>rank 40 iram choudhary</t>
+  </si>
+  <si>
+    <t>rank 7 aayushi bansal</t>
   </si>
 </sst>
 </file>
@@ -202,7 +196,7 @@
     </font>
     <font>
       <sz val="16"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Mistral"/>
       <family val="4"/>
     </font>
@@ -233,12 +227,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -550,7 +551,7 @@
   <dimension ref="A1:A13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.5703125" customWidth="1"/>
     <col min="2" max="2" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -561,17 +562,17 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
@@ -591,32 +592,32 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -629,9 +630,9 @@
   <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35" style="1" customWidth="1"/>
+    <col min="1" max="1" width="40.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -647,7 +648,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2" s="1">
         <v>2021</v>
@@ -658,191 +659,195 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B3" s="1">
         <v>2022</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B4" s="1">
         <v>2023</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B5" s="1">
         <v>2024</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B6" s="1">
         <v>2025</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B7" s="1">
         <v>2026</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" ht="21.75" x14ac:dyDescent="0.4">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="21.75" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
-        <v>37</v>
+      <c r="A23" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
-        <v>38</v>
+      <c r="A24" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
-        <v>39</v>
+      <c r="A25" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
-        <v>40</v>
+      <c r="A26" s="2" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
-        <v>41</v>
+      <c r="A27" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
-        <v>42</v>
+      <c r="A28" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" s="1" t="s">
-        <v>43</v>
+      <c r="A29" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" s="1" t="s">
-        <v>44</v>
+      <c r="A30" s="2" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" s="1" t="s">
-        <v>45</v>
+      <c r="A31" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" s="1" t="s">
-        <v>46</v>
+      <c r="A32" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C33"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:A32 A34:A1048576">
+  <conditionalFormatting sqref="A1 A34:A1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1 A33:A1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>